<commit_message>
Initial commit - CEO dashboard project
</commit_message>
<xml_diff>
--- a/excel-imports/student_performance.xlsx
+++ b/excel-imports/student_performance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\school-ceo-dashboard review 1\school-ceo-dashboard\excel-imports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BCB8823-CC9A-419E-8287-185B0E2A3CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F52D8B4-9BFC-41B3-8F7F-728E541956E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -568,10 +568,10 @@
         <v>0.74</v>
       </c>
       <c r="E2" s="1">
-        <v>0.85</v>
+        <v>0.87</v>
       </c>
       <c r="F2" s="1">
-        <v>0.76</v>
+        <v>0.89</v>
       </c>
       <c r="G2" s="1">
         <v>0.85</v>

</xml_diff>